<commit_message>
Upgrade 7B213 journal lines in EVID overlay to CITED (ledger reconciled)
The 34 NA7B213 immunisation recode lines move INTAKE-HELD -> CITED now that the
Parks 7B213 ledger reconciles to the manifest exactly and the immunisation
journal source is held. EVID overlay status: 171 PRESENT, 34 CITED, 48 PRESENT*,
114 CONSOLIDATED, 0 deficient. Manifest strict-verify PASS.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sv2n4PfmaM4LstEnSuMyfB
</commit_message>
<xml_diff>
--- a/00_Live_Recode_Journal_EVID_17-Jun-2026.xlsx
+++ b/00_Live_Recode_Journal_EVID_17-Jun-2026.xlsx
@@ -518,7 +518,7 @@
     <row r="2" ht="15" customHeight="1" s="16">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Batch CN-23167. 367 lines (333 prior + 34 NA7B213 added 17-Jun, 34 NA7B213 source held as intake, not yet sighted per line), batch nets $0.00. EVID = unique evidence-source identifier (see Evidence Source Register). EvStatus = strongest sighting held. Deficient=Y means no held source.</t>
+          <t>Batch CN-23167. 367 lines (333 prior + 34 NA7B213 added 17-Jun, 34 NA7B213 cited to the Parks 7B213 ledger (reconciles exact) + immunisation journal), batch nets $0.00. EVID = unique evidence-source identifier (see Evidence Source Register). EvStatus = strongest sighting held. Deficient=Y means no held source.</t>
         </is>
       </c>
     </row>
@@ -21552,12 +21552,12 @@
       </c>
       <c r="J338" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K338" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L338" s="27" t="inlineStr">
@@ -21567,7 +21567,7 @@
       </c>
       <c r="M338" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -21615,12 +21615,12 @@
       </c>
       <c r="J339" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K339" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L339" s="27" t="inlineStr">
@@ -21630,7 +21630,7 @@
       </c>
       <c r="M339" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -21678,12 +21678,12 @@
       </c>
       <c r="J340" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K340" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L340" s="27" t="inlineStr">
@@ -21693,7 +21693,7 @@
       </c>
       <c r="M340" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -21741,12 +21741,12 @@
       </c>
       <c r="J341" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K341" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L341" s="27" t="inlineStr">
@@ -21756,7 +21756,7 @@
       </c>
       <c r="M341" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -21804,12 +21804,12 @@
       </c>
       <c r="J342" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K342" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L342" s="27" t="inlineStr">
@@ -21819,7 +21819,7 @@
       </c>
       <c r="M342" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -21867,12 +21867,12 @@
       </c>
       <c r="J343" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K343" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L343" s="27" t="inlineStr">
@@ -21882,7 +21882,7 @@
       </c>
       <c r="M343" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -21930,12 +21930,12 @@
       </c>
       <c r="J344" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K344" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L344" s="27" t="inlineStr">
@@ -21945,7 +21945,7 @@
       </c>
       <c r="M344" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -21993,12 +21993,12 @@
       </c>
       <c r="J345" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K345" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L345" s="27" t="inlineStr">
@@ -22008,7 +22008,7 @@
       </c>
       <c r="M345" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -22056,12 +22056,12 @@
       </c>
       <c r="J346" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K346" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L346" s="27" t="inlineStr">
@@ -22071,7 +22071,7 @@
       </c>
       <c r="M346" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -22119,12 +22119,12 @@
       </c>
       <c r="J347" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K347" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L347" s="27" t="inlineStr">
@@ -22134,7 +22134,7 @@
       </c>
       <c r="M347" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -22182,12 +22182,12 @@
       </c>
       <c r="J348" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K348" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L348" s="27" t="inlineStr">
@@ -22197,7 +22197,7 @@
       </c>
       <c r="M348" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -22245,12 +22245,12 @@
       </c>
       <c r="J349" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K349" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L349" s="27" t="inlineStr">
@@ -22260,7 +22260,7 @@
       </c>
       <c r="M349" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -22308,12 +22308,12 @@
       </c>
       <c r="J350" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K350" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L350" s="27" t="inlineStr">
@@ -22323,7 +22323,7 @@
       </c>
       <c r="M350" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -22371,12 +22371,12 @@
       </c>
       <c r="J351" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K351" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L351" s="27" t="inlineStr">
@@ -22386,7 +22386,7 @@
       </c>
       <c r="M351" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -22434,12 +22434,12 @@
       </c>
       <c r="J352" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K352" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L352" s="27" t="inlineStr">
@@ -22449,7 +22449,7 @@
       </c>
       <c r="M352" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -22497,12 +22497,12 @@
       </c>
       <c r="J353" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K353" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L353" s="27" t="inlineStr">
@@ -22512,7 +22512,7 @@
       </c>
       <c r="M353" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -22560,12 +22560,12 @@
       </c>
       <c r="J354" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K354" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L354" s="27" t="inlineStr">
@@ -22575,7 +22575,7 @@
       </c>
       <c r="M354" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -22623,12 +22623,12 @@
       </c>
       <c r="J355" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K355" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L355" s="27" t="inlineStr">
@@ -22638,7 +22638,7 @@
       </c>
       <c r="M355" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -22686,12 +22686,12 @@
       </c>
       <c r="J356" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K356" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L356" s="27" t="inlineStr">
@@ -22701,7 +22701,7 @@
       </c>
       <c r="M356" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -22749,12 +22749,12 @@
       </c>
       <c r="J357" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K357" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L357" s="27" t="inlineStr">
@@ -22764,7 +22764,7 @@
       </c>
       <c r="M357" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -22812,12 +22812,12 @@
       </c>
       <c r="J358" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K358" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L358" s="27" t="inlineStr">
@@ -22827,7 +22827,7 @@
       </c>
       <c r="M358" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -22875,12 +22875,12 @@
       </c>
       <c r="J359" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K359" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L359" s="27" t="inlineStr">
@@ -22890,7 +22890,7 @@
       </c>
       <c r="M359" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -22938,12 +22938,12 @@
       </c>
       <c r="J360" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K360" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L360" s="27" t="inlineStr">
@@ -22953,7 +22953,7 @@
       </c>
       <c r="M360" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -23001,12 +23001,12 @@
       </c>
       <c r="J361" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K361" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L361" s="27" t="inlineStr">
@@ -23016,7 +23016,7 @@
       </c>
       <c r="M361" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -23064,12 +23064,12 @@
       </c>
       <c r="J362" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K362" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L362" s="27" t="inlineStr">
@@ -23079,7 +23079,7 @@
       </c>
       <c r="M362" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -23127,12 +23127,12 @@
       </c>
       <c r="J363" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K363" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L363" s="27" t="inlineStr">
@@ -23142,7 +23142,7 @@
       </c>
       <c r="M363" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -23190,12 +23190,12 @@
       </c>
       <c r="J364" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K364" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L364" s="27" t="inlineStr">
@@ -23205,7 +23205,7 @@
       </c>
       <c r="M364" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -23253,12 +23253,12 @@
       </c>
       <c r="J365" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K365" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L365" s="27" t="inlineStr">
@@ -23268,7 +23268,7 @@
       </c>
       <c r="M365" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -23316,12 +23316,12 @@
       </c>
       <c r="J366" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K366" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L366" s="27" t="inlineStr">
@@ -23331,7 +23331,7 @@
       </c>
       <c r="M366" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -23379,12 +23379,12 @@
       </c>
       <c r="J367" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K367" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L367" s="27" t="inlineStr">
@@ -23394,7 +23394,7 @@
       </c>
       <c r="M367" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -23442,12 +23442,12 @@
       </c>
       <c r="J368" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K368" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L368" s="27" t="inlineStr">
@@ -23457,7 +23457,7 @@
       </c>
       <c r="M368" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -23505,12 +23505,12 @@
       </c>
       <c r="J369" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K369" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L369" s="27" t="inlineStr">
@@ -23520,7 +23520,7 @@
       </c>
       <c r="M369" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -23568,12 +23568,12 @@
       </c>
       <c r="J370" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K370" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L370" s="27" t="inlineStr">
@@ -23583,7 +23583,7 @@
       </c>
       <c r="M370" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>
@@ -23631,12 +23631,12 @@
       </c>
       <c r="J371" s="20" t="inlineStr">
         <is>
-          <t>EVID-7B213-src</t>
+          <t>EVID-7B213-ledger</t>
         </is>
       </c>
       <c r="K371" s="27" t="inlineStr">
         <is>
-          <t>INTAKE-HELD</t>
+          <t>CITED</t>
         </is>
       </c>
       <c r="L371" s="27" t="inlineStr">
@@ -23646,7 +23646,7 @@
       </c>
       <c r="M371" s="21" t="inlineStr">
         <is>
-          <t>_Sources_16-Jun-2026/NA7B213_Intake/Internal_Medical.XLSM (whole-branch immunisation recharge; internal charge, no per-line external invoice; not yet sighted per officer line)</t>
+          <t>NA7B213_Ledger_4090000_18-Jun-2026.xlsx (70 lines reconcile $4,861.70 exact) + Internal Immunisation Services Journal (per-officer/vaccine source)</t>
         </is>
       </c>
     </row>

</xml_diff>